<commit_message>
Created gantt chart (optimised) - not integrated with the main app yet
Debugging required: stockpile profile report, blend_ID
</commit_message>
<xml_diff>
--- a/blendmaster_OOP/output/build_report_2024-11-28_06-00.xlsx
+++ b/blendmaster_OOP/output/build_report_2024-11-28_06-00.xlsx
@@ -9607,22 +9607,22 @@
         <v>45624.68828857363</v>
       </c>
       <c r="J173" t="n">
-        <v>48826.69402005</v>
+        <v>47345.61978727223</v>
       </c>
       <c r="K173" t="n">
-        <v>58.1226909501456</v>
+        <v>58.12277855867986</v>
       </c>
       <c r="L173" t="n">
-        <v>4.573884320919685</v>
+        <v>4.573725508275982</v>
       </c>
       <c r="M173" t="n">
-        <v>3.330814804226851</v>
+        <v>3.330931224743555</v>
       </c>
       <c r="N173" t="n">
-        <v>0.1066907922988864</v>
+        <v>0.1066986626157106</v>
       </c>
       <c r="O173" t="n">
-        <v>0.03821646236709458</v>
+        <v>0.03822029321187685</v>
       </c>
     </row>
     <row r="174">

</xml_diff>